<commit_message>
Clarify Reynolds-number metadata formulas
Replace descriptive Reynolds-number basis entries with explicit calculation formulas across the study metadata, including pointwise conversions and assumptions. Update the Excel workbook to match the CSV.
</commit_message>
<xml_diff>
--- a/(Troposkein) Research Papers/!management/metadata_troposkein.xlsx
+++ b/(Troposkein) Research Papers/!management/metadata_troposkein.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="R4efb7fe688af44f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Re_D Calculations" sheetId="2" r:id="R50b8b95712c44a67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="R35a5abfcc1d741cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Re_D Calculations" sheetId="2" r:id="R42922a3cc06f4635"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -288,7 +288,7 @@
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="48" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="22" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="22" hidden="0" customWidth="1"/>
@@ -388,7 +388,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P2" s="4" t="str">
-        <x:v>Pointwise; geometry required</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q2" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -429,7 +429,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P3" s="4" t="str">
-        <x:v>Pointwise; geometry required</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q3" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -470,7 +470,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P4" s="4" t="str">
-        <x:v>Pointwise; geometry required</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q4" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -511,7 +511,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P5" s="4" t="str">
-        <x:v>Pointwise; geometry required</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q5" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -581,7 +581,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P7" s="4" t="str">
-        <x:v>estimated pointwise; measured U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.51*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q7" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -653,7 +653,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P9" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q9" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -702,7 +702,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P10" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q10" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -751,7 +751,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P11" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q11" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -800,7 +800,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P12" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q12" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -849,7 +849,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P13" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q13" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -898,7 +898,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P14" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q14" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -947,7 +947,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P15" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q15" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -996,7 +996,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P16" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q16" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1045,7 +1045,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P17" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q17" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1094,7 +1094,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P18" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q18" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1143,7 +1143,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P19" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q19" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1192,7 +1192,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P20" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q20" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1241,7 +1241,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P21" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q21" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1290,7 +1290,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P22" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q22" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1339,7 +1339,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P23" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q23" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1388,7 +1388,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P24" s="4" t="str">
-        <x:v>estimated pointwise; nominal rpm and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*Re_rot/(cToR*TSR)</x:v>
       </x:c>
       <x:c r="Q24" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1439,7 +1439,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P25" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q25" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1490,7 +1490,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P26" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q26" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1541,7 +1541,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P27" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q27" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1592,7 +1592,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P28" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q28" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1643,7 +1643,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P29" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q29" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1694,7 +1694,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P30" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q30" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1745,7 +1745,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P31" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q31" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1796,7 +1796,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P32" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q32" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1847,7 +1847,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P33" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q33" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1898,7 +1898,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P34" s="4" t="str">
-        <x:v>estimated; fixed U; assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 1.9596*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q34" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -1968,7 +1968,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P36" s="4" t="str">
-        <x:v>estimated pointwise from Table I wind speed; nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 4.2672*U_m_s/0.000015</x:v>
       </x:c>
       <x:c r="Q36" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2038,7 +2038,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P38" s="4" t="str">
-        <x:v>approximate pointwise route; nominal D=5 m and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*(2*pi*RPM/60)*2.5^2/(0.000015*TSR)</x:v>
       </x:c>
       <x:c r="Q38" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2081,7 +2081,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P39" s="4" t="str">
-        <x:v>approximate pointwise route; nominal D=5 m and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*(2*pi*RPM/60)*2.5^2/(0.000015*TSR)</x:v>
       </x:c>
       <x:c r="Q39" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2124,7 +2124,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P40" s="4" t="str">
-        <x:v>approximate pointwise route; nominal D=5 m and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*(2*pi*RPM/60)*2.5^2/(0.000015*TSR)</x:v>
       </x:c>
       <x:c r="Q40" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2167,7 +2167,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P41" s="4" t="str">
-        <x:v>approximate pointwise route; nominal D=5 m and assumed nu=1.50e-5 m2/s</x:v>
+        <x:v>Re_D = 2*(2*pi*RPM/60)*2.5^2/(0.000015*TSR)</x:v>
       </x:c>
       <x:c r="Q41" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2235,7 +2235,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P43" s="4" t="str">
-        <x:v>Pointwise; uses source rounded cToR</x:v>
+        <x:v>Re_D = 2*Re_rot/(0.067*TSR)</x:v>
       </x:c>
       <x:c r="Q43" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2280,7 +2280,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P44" s="4" t="str">
-        <x:v>Pointwise; uses source rounded cToR</x:v>
+        <x:v>Re_D = 2*Re_rot/(0.067*TSR)</x:v>
       </x:c>
       <x:c r="Q44" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2325,7 +2325,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P45" s="4" t="str">
-        <x:v>Pointwise; uses source rounded cToR</x:v>
+        <x:v>Re_D = 2*Re_rot/(0.067*TSR)</x:v>
       </x:c>
       <x:c r="Q45" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2370,7 +2370,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P46" s="4" t="str">
-        <x:v>Pointwise; uses source rounded cToR</x:v>
+        <x:v>Re_D = 2*Re_rot/(0.067*TSR)</x:v>
       </x:c>
       <x:c r="Q46" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>
@@ -2415,7 +2415,7 @@
         <x:v>air</x:v>
       </x:c>
       <x:c r="P47" s="4" t="str">
-        <x:v>Pointwise; uses source rounded cToR</x:v>
+        <x:v>Re_D = 2*Re_rot/(0.067*TSR)</x:v>
       </x:c>
       <x:c r="Q47" s="4" t="str">
         <x:v>Not assigned; no uniform physical pitch verified</x:v>

</xml_diff>